<commit_message>
Fixes incorrect output CSV structure in BCF
</commit_message>
<xml_diff>
--- a/InputData/web-app/BCF/BTU Conversion Factors.xlsx
+++ b/InputData/web-app/BCF/BTU Conversion Factors.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Olivia Ashmoore\Documents\EPS_Models by Region\United States\us-eps\InputData\web-app\BCF\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\web-app\BCF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AD158D4-4564-4341-A436-73B4713E8C38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{142D0A21-AD9A-446A-9902-4DB5430B75D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23385" yWindow="1695" windowWidth="20625" windowHeight="15075" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -19317,6 +19317,9 @@
       <c r="AA1">
         <v>2049</v>
       </c>
+      <c r="AB1">
+        <v>2050</v>
+      </c>
     </row>
     <row r="2" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
@@ -19400,7 +19403,7 @@
       <c r="AA2">
         <v>0</v>
       </c>
-      <c r="AC2">
+      <c r="AB2">
         <v>0</v>
       </c>
     </row>
@@ -19486,7 +19489,7 @@
       <c r="AA3">
         <v>0</v>
       </c>
-      <c r="AC3">
+      <c r="AB3">
         <v>0</v>
       </c>
     </row>
@@ -19598,11 +19601,11 @@
         <f>'AEO Table 73'!AB32*10^6/gal_per_barrel</f>
         <v>119586.72886803036</v>
       </c>
-      <c r="AB4" s="4"/>
-      <c r="AC4" s="4">
-        <f>'AEO Table 73'!AD32*10^6/gal_per_barrel</f>
-        <v>-5.0246875992093498</v>
-      </c>
+      <c r="AB4" s="4">
+        <f>'AEO Table 73'!AC32*10^6/gal_per_barrel</f>
+        <v>119565.13495672317</v>
+      </c>
+      <c r="AC4" s="4"/>
     </row>
     <row r="5" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
@@ -19712,11 +19715,11 @@
         <f>'AEO Table 73'!AB19*10^6/gal_per_barrel</f>
         <v>138690.47164916992</v>
       </c>
-      <c r="AB5" s="4"/>
-      <c r="AC5" s="4">
-        <f>'AEO Table 73'!AD19*10^6/gal_per_barrel</f>
-        <v>0</v>
-      </c>
+      <c r="AB5" s="4">
+        <f>'AEO Table 73'!AC19*10^6/gal_per_barrel</f>
+        <v>138690.47164916992</v>
+      </c>
+      <c r="AC5" s="4"/>
     </row>
     <row r="6" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
@@ -19800,7 +19803,7 @@
       <c r="AA6">
         <v>0</v>
       </c>
-      <c r="AC6">
+      <c r="AB6">
         <v>0</v>
       </c>
     </row>
@@ -19886,7 +19889,7 @@
       <c r="AA7">
         <v>0</v>
       </c>
-      <c r="AC7">
+      <c r="AB7">
         <v>0</v>
       </c>
     </row>
@@ -19998,11 +20001,11 @@
         <f>'AEO Table 73'!AB30*10^6/gal_per_barrel</f>
         <v>135000.0018165225</v>
       </c>
-      <c r="AB8" s="4"/>
-      <c r="AC8" s="4">
-        <f>'AEO Table 73'!AD30*10^6/gal_per_barrel</f>
-        <v>0</v>
-      </c>
+      <c r="AB8" s="4">
+        <f>'AEO Table 73'!AC30*10^6/gal_per_barrel</f>
+        <v>135000.0018165225</v>
+      </c>
+      <c r="AC8" s="4"/>
     </row>
     <row r="9" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
@@ -20086,7 +20089,7 @@
       <c r="AA9">
         <v>0</v>
       </c>
-      <c r="AC9">
+      <c r="AB9">
         <v>0</v>
       </c>
     </row>
@@ -20172,7 +20175,7 @@
       <c r="AA10">
         <v>0</v>
       </c>
-      <c r="AC10">
+      <c r="AB10">
         <v>0</v>
       </c>
     </row>
@@ -20258,7 +20261,7 @@
       <c r="AA11">
         <v>0</v>
       </c>
-      <c r="AC11">
+      <c r="AB11">
         <v>0</v>
       </c>
     </row>

</xml_diff>